<commit_message>
Updated CHN_grids_kan10 model - 2026-06-26 13:57
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN_grids_kan10/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_CHN_grids_kan10/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr updateLinks="never"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN_grids_kan10\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FFA8710F-2F7A-4ADB-8533-D6C692C06817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{49613383-CF92-490D-89FF-2EF1742B8846}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="135">
   <si>
     <t>PSET_PN</t>
   </si>
@@ -292,6 +292,9 @@
     <t>coal,oil,bioenergy</t>
   </si>
   <si>
+    <t>AF</t>
+  </si>
+  <si>
     <t>~replicateinregions</t>
   </si>
   <si>
@@ -301,85 +304,145 @@
     <t>indesc</t>
   </si>
   <si>
+    <t>IND</t>
+  </si>
+  <si>
+    <t>en_gas_ccgt,en_gas_turbine,en_gas_chp,en_gas_fuelcell,en_gas_ccs,en_coal_subcritical,en_coal_supercritical,en_coal_ultrasupercritical,en_coal_igcc,en_coal_ccs,en_coal_igcc_ccs,en_coal_oxyfuel_ccs,en_nuclear,en_nuclear_smr,en_biomass,en_biomass_cofiring,en_biomass_chp,en_biomass_ccs,en_geothermal</t>
+  </si>
+  <si>
+    <t>w420797421-765_IND</t>
+  </si>
+  <si>
+    <t>at grid node - w420797421-765_IND</t>
+  </si>
+  <si>
+    <t>w759521252-765_IND</t>
+  </si>
+  <si>
+    <t>at grid node - w759521252-765_IND</t>
+  </si>
+  <si>
+    <t>w688672711-765_IND</t>
+  </si>
+  <si>
+    <t>at grid node - w688672711-765_IND</t>
+  </si>
+  <si>
+    <t>w372701897-765_IND</t>
+  </si>
+  <si>
+    <t>at grid node - w372701897-765_IND</t>
+  </si>
+  <si>
+    <t>w1143180503-765_IND</t>
+  </si>
+  <si>
+    <t>at grid node - w1143180503-765_IND</t>
+  </si>
+  <si>
+    <t>IN684-765_IND</t>
+  </si>
+  <si>
+    <t>at grid node - IN684-765_IND</t>
+  </si>
+  <si>
+    <t>w331275940-765_IND</t>
+  </si>
+  <si>
+    <t>at grid node - w331275940-765_IND</t>
+  </si>
+  <si>
+    <t>EN_STG8hbNREL,EN_STG4hbNREL</t>
+  </si>
+  <si>
+    <t>w203673991-400_IND</t>
+  </si>
+  <si>
+    <t>at grid node - w203673991-400_IND</t>
+  </si>
+  <si>
+    <t>e_demand,ev_battery,H2prd_Elc_PEM,H2prd_Elc_ALK</t>
+  </si>
+  <si>
+    <t>pset_pn</t>
+  </si>
+  <si>
+    <t>-*cofiring*</t>
+  </si>
+  <si>
+    <t>-EFF</t>
+  </si>
+  <si>
+    <t>en_biomass_cofiring*,en_geothermal*</t>
+  </si>
+  <si>
     <t>CHN</t>
   </si>
   <si>
+    <t>w966809494-500_CHN</t>
+  </si>
+  <si>
+    <t>at grid node - w966809494-500_CHN</t>
+  </si>
+  <si>
+    <t>w1347514254-500_CHN</t>
+  </si>
+  <si>
+    <t>at grid node - w1347514254-500_CHN</t>
+  </si>
+  <si>
+    <t>w462823764-500_CHN</t>
+  </si>
+  <si>
+    <t>at grid node - w462823764-500_CHN</t>
+  </si>
+  <si>
     <t>w148727570-500_CHN</t>
   </si>
   <si>
     <t>at grid node - w148727570-500_CHN</t>
   </si>
   <si>
-    <t>Bioenergy + CCUS,Bioenergy - Large scale unit,CCGT,CCGT + CCS,Coal + CCS,Gas turbine,IGCC,IGCC + CCS,Nuclear large,Oxyfuel + CCS,Steam Coal - SUBCRITICAL,Steam Coal - SUPERCRITICAL,Steam Coal - ULTRASUPERCRITICAL</t>
-  </si>
-  <si>
-    <t>w462823764-500_CHN</t>
-  </si>
-  <si>
-    <t>at grid node - w462823764-500_CHN</t>
-  </si>
-  <si>
-    <t>w966809494-500_CHN</t>
-  </si>
-  <si>
-    <t>at grid node - w966809494-500_CHN</t>
+    <t>w127871762-500_CHN</t>
+  </si>
+  <si>
+    <t>at grid node - w127871762-500_CHN</t>
+  </si>
+  <si>
+    <t>CN7501-500_CHN</t>
+  </si>
+  <si>
+    <t>at grid node - CN7501-500_CHN</t>
+  </si>
+  <si>
+    <t>w858207240-500_CHN</t>
+  </si>
+  <si>
+    <t>at grid node - w858207240-500_CHN</t>
+  </si>
+  <si>
+    <t>w568247904-750_CHN</t>
+  </si>
+  <si>
+    <t>at grid node - w568247904-750_CHN</t>
+  </si>
+  <si>
+    <t>w178865921-500_CHN</t>
+  </si>
+  <si>
+    <t>at grid node - w178865921-500_CHN</t>
+  </si>
+  <si>
+    <t>w251393861-500_CHN</t>
+  </si>
+  <si>
+    <t>at grid node - w251393861-500_CHN</t>
   </si>
   <si>
     <t>w899674815-750_CHN</t>
   </si>
   <si>
     <t>at grid node - w899674815-750_CHN</t>
-  </si>
-  <si>
-    <t>w251393861-500_CHN</t>
-  </si>
-  <si>
-    <t>at grid node - w251393861-500_CHN</t>
-  </si>
-  <si>
-    <t>w1347514254-500_CHN</t>
-  </si>
-  <si>
-    <t>at grid node - w1347514254-500_CHN</t>
-  </si>
-  <si>
-    <t>w127871762-500_CHN</t>
-  </si>
-  <si>
-    <t>at grid node - w127871762-500_CHN</t>
-  </si>
-  <si>
-    <t>w178865921-500_CHN</t>
-  </si>
-  <si>
-    <t>at grid node - w178865921-500_CHN</t>
-  </si>
-  <si>
-    <t>w858207240-500_CHN</t>
-  </si>
-  <si>
-    <t>at grid node - w858207240-500_CHN</t>
-  </si>
-  <si>
-    <t>CN7501-500_CHN</t>
-  </si>
-  <si>
-    <t>at grid node - CN7501-500_CHN</t>
-  </si>
-  <si>
-    <t>w568247904-750_CHN</t>
-  </si>
-  <si>
-    <t>at grid node - w568247904-750_CHN</t>
-  </si>
-  <si>
-    <t>EN_Hydro_CHN-1,EN_Hydro_CHN-2,EN_Hydro_CHN-3</t>
-  </si>
-  <si>
-    <t>EN_STG8hbNREL,EN_STG4hbNREL</t>
-  </si>
-  <si>
-    <t>e_demand,ev_battery,H2prd_Elc_PEM,H2prd_Elc_ALK</t>
   </si>
 </sst>
 </file>
@@ -707,15 +770,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{268E9BAB-B98F-4B82-9042-51EABC9ED525}">
-  <dimension ref="B3:T21"/>
+  <dimension ref="B3:O26"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="3" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
         <v>21</v>
       </c>
@@ -723,7 +786,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
         <v>59</v>
       </c>
@@ -731,29 +794,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="L9" t="s">
-        <v>84</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.45">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
         <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E10" t="s">
         <v>21</v>
@@ -762,10 +822,10 @@
         <v>33</v>
       </c>
       <c r="H10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J10" t="s">
         <v>21</v>
@@ -774,563 +834,609 @@
         <v>33</v>
       </c>
       <c r="M10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O10" t="s">
         <v>21</v>
       </c>
-      <c r="Q10" t="s">
-        <v>33</v>
-      </c>
-      <c r="R10" t="s">
-        <v>85</v>
-      </c>
-      <c r="S10" t="s">
-        <v>86</v>
-      </c>
-      <c r="T10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.45">
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="C11" t="s">
+        <v>113</v>
+      </c>
+      <c r="D11" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11" t="s">
+        <v>112</v>
+      </c>
+      <c r="H11" t="s">
+        <v>113</v>
+      </c>
+      <c r="I11" t="s">
+        <v>114</v>
+      </c>
+      <c r="J11" t="s">
+        <v>104</v>
+      </c>
+      <c r="L11" t="s">
+        <v>112</v>
+      </c>
+      <c r="M11" t="s">
+        <v>121</v>
+      </c>
+      <c r="N11" t="s">
+        <v>122</v>
+      </c>
+      <c r="O11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B12" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" t="s">
+        <v>116</v>
+      </c>
+      <c r="E12" t="s">
+        <v>89</v>
+      </c>
+      <c r="G12" t="s">
+        <v>112</v>
+      </c>
+      <c r="H12" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" t="s">
+        <v>116</v>
+      </c>
+      <c r="J12" t="s">
+        <v>104</v>
+      </c>
+      <c r="L12" t="s">
+        <v>112</v>
+      </c>
+      <c r="M12" t="s">
+        <v>119</v>
+      </c>
+      <c r="N12" t="s">
+        <v>120</v>
+      </c>
+      <c r="O12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B13" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" t="s">
+        <v>117</v>
+      </c>
+      <c r="D13" t="s">
+        <v>118</v>
+      </c>
+      <c r="E13" t="s">
+        <v>89</v>
+      </c>
+      <c r="G13" t="s">
+        <v>112</v>
+      </c>
+      <c r="H13" t="s">
+        <v>117</v>
+      </c>
+      <c r="I13" t="s">
+        <v>118</v>
+      </c>
+      <c r="J13" t="s">
+        <v>104</v>
+      </c>
+      <c r="L13" t="s">
+        <v>112</v>
+      </c>
+      <c r="M13" t="s">
+        <v>129</v>
+      </c>
+      <c r="N13" t="s">
+        <v>130</v>
+      </c>
+      <c r="O13" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B14" t="s">
+        <v>112</v>
+      </c>
+      <c r="C14" t="s">
+        <v>119</v>
+      </c>
+      <c r="D14" t="s">
+        <v>120</v>
+      </c>
+      <c r="E14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G14" t="s">
+        <v>112</v>
+      </c>
+      <c r="H14" t="s">
+        <v>119</v>
+      </c>
+      <c r="I14" t="s">
+        <v>120</v>
+      </c>
+      <c r="J14" t="s">
+        <v>104</v>
+      </c>
+      <c r="L14" t="s">
+        <v>112</v>
+      </c>
+      <c r="M14" t="s">
+        <v>131</v>
+      </c>
+      <c r="N14" t="s">
+        <v>132</v>
+      </c>
+      <c r="O14" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B15" t="s">
+        <v>112</v>
+      </c>
+      <c r="C15" t="s">
+        <v>121</v>
+      </c>
+      <c r="D15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" t="s">
+        <v>112</v>
+      </c>
+      <c r="H15" t="s">
+        <v>121</v>
+      </c>
+      <c r="I15" t="s">
+        <v>122</v>
+      </c>
+      <c r="J15" t="s">
+        <v>104</v>
+      </c>
+      <c r="L15" t="s">
+        <v>112</v>
+      </c>
+      <c r="M15" t="s">
+        <v>117</v>
+      </c>
+      <c r="N15" t="s">
+        <v>118</v>
+      </c>
+      <c r="O15" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B16" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" t="s">
+        <v>123</v>
+      </c>
+      <c r="D16" t="s">
+        <v>124</v>
+      </c>
+      <c r="E16" t="s">
+        <v>89</v>
+      </c>
+      <c r="G16" t="s">
+        <v>112</v>
+      </c>
+      <c r="H16" t="s">
+        <v>123</v>
+      </c>
+      <c r="I16" t="s">
+        <v>124</v>
+      </c>
+      <c r="J16" t="s">
+        <v>104</v>
+      </c>
+      <c r="L16" t="s">
+        <v>112</v>
+      </c>
+      <c r="M16" t="s">
+        <v>115</v>
+      </c>
+      <c r="N16" t="s">
+        <v>116</v>
+      </c>
+      <c r="O16" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B17" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" t="s">
+        <v>125</v>
+      </c>
+      <c r="D17" t="s">
+        <v>126</v>
+      </c>
+      <c r="E17" t="s">
+        <v>89</v>
+      </c>
+      <c r="G17" t="s">
+        <v>112</v>
+      </c>
+      <c r="H17" t="s">
+        <v>125</v>
+      </c>
+      <c r="I17" t="s">
+        <v>126</v>
+      </c>
+      <c r="J17" t="s">
+        <v>104</v>
+      </c>
+      <c r="L17" t="s">
+        <v>112</v>
+      </c>
+      <c r="M17" t="s">
+        <v>125</v>
+      </c>
+      <c r="N17" t="s">
+        <v>126</v>
+      </c>
+      <c r="O17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B18" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" t="s">
+        <v>127</v>
+      </c>
+      <c r="D18" t="s">
+        <v>128</v>
+      </c>
+      <c r="E18" t="s">
+        <v>89</v>
+      </c>
+      <c r="G18" t="s">
+        <v>112</v>
+      </c>
+      <c r="H18" t="s">
+        <v>127</v>
+      </c>
+      <c r="I18" t="s">
+        <v>128</v>
+      </c>
+      <c r="J18" t="s">
+        <v>104</v>
+      </c>
+      <c r="L18" t="s">
+        <v>112</v>
+      </c>
+      <c r="M18" t="s">
+        <v>133</v>
+      </c>
+      <c r="N18" t="s">
+        <v>134</v>
+      </c>
+      <c r="O18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C19" t="s">
+        <v>129</v>
+      </c>
+      <c r="D19" t="s">
+        <v>130</v>
+      </c>
+      <c r="E19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G19" t="s">
+        <v>112</v>
+      </c>
+      <c r="H19" t="s">
+        <v>129</v>
+      </c>
+      <c r="I19" t="s">
+        <v>130</v>
+      </c>
+      <c r="J19" t="s">
+        <v>104</v>
+      </c>
+      <c r="L19" t="s">
+        <v>112</v>
+      </c>
+      <c r="M19" t="s">
+        <v>113</v>
+      </c>
+      <c r="N19" t="s">
+        <v>114</v>
+      </c>
+      <c r="O19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="20" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B20" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" t="s">
+        <v>131</v>
+      </c>
+      <c r="D20" t="s">
+        <v>132</v>
+      </c>
+      <c r="E20" t="s">
+        <v>89</v>
+      </c>
+      <c r="G20" t="s">
+        <v>112</v>
+      </c>
+      <c r="H20" t="s">
+        <v>131</v>
+      </c>
+      <c r="I20" t="s">
+        <v>132</v>
+      </c>
+      <c r="J20" t="s">
+        <v>104</v>
+      </c>
+      <c r="L20" t="s">
+        <v>112</v>
+      </c>
+      <c r="M20" t="s">
+        <v>123</v>
+      </c>
+      <c r="N20" t="s">
+        <v>124</v>
+      </c>
+      <c r="O20" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B21" t="s">
         <v>88</v>
       </c>
-      <c r="D11" t="s">
+      <c r="C21" t="s">
+        <v>94</v>
+      </c>
+      <c r="D21" t="s">
+        <v>95</v>
+      </c>
+      <c r="E21" t="s">
         <v>89</v>
       </c>
-      <c r="E11" t="s">
+      <c r="G21" t="s">
+        <v>112</v>
+      </c>
+      <c r="H21" t="s">
+        <v>133</v>
+      </c>
+      <c r="I21" t="s">
+        <v>134</v>
+      </c>
+      <c r="J21" t="s">
+        <v>104</v>
+      </c>
+      <c r="L21" t="s">
+        <v>88</v>
+      </c>
+      <c r="M21" t="s">
         <v>90</v>
       </c>
-      <c r="G11" t="s">
-        <v>87</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="N21" t="s">
+        <v>91</v>
+      </c>
+      <c r="O21" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B22" t="s">
+        <v>88</v>
+      </c>
+      <c r="C22" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" t="s">
+        <v>97</v>
+      </c>
+      <c r="E22" t="s">
+        <v>89</v>
+      </c>
+      <c r="G22" t="s">
+        <v>88</v>
+      </c>
+      <c r="H22" t="s">
+        <v>96</v>
+      </c>
+      <c r="I22" t="s">
+        <v>97</v>
+      </c>
+      <c r="J22" t="s">
+        <v>104</v>
+      </c>
+      <c r="L22" t="s">
+        <v>88</v>
+      </c>
+      <c r="M22" t="s">
+        <v>94</v>
+      </c>
+      <c r="N22" t="s">
+        <v>95</v>
+      </c>
+      <c r="O22" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B23" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D23" t="s">
+        <v>99</v>
+      </c>
+      <c r="E23" t="s">
+        <v>89</v>
+      </c>
+      <c r="G23" t="s">
+        <v>88</v>
+      </c>
+      <c r="H23" t="s">
+        <v>98</v>
+      </c>
+      <c r="I23" t="s">
+        <v>99</v>
+      </c>
+      <c r="J23" t="s">
+        <v>104</v>
+      </c>
+      <c r="L23" t="s">
+        <v>88</v>
+      </c>
+      <c r="M23" t="s">
+        <v>92</v>
+      </c>
+      <c r="N23" t="s">
+        <v>93</v>
+      </c>
+      <c r="O23" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="24" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24" t="s">
+        <v>100</v>
+      </c>
+      <c r="D24" t="s">
+        <v>101</v>
+      </c>
+      <c r="E24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G24" t="s">
+        <v>88</v>
+      </c>
+      <c r="H24" t="s">
+        <v>100</v>
+      </c>
+      <c r="I24" t="s">
+        <v>101</v>
+      </c>
+      <c r="J24" t="s">
+        <v>104</v>
+      </c>
+      <c r="L24" t="s">
+        <v>88</v>
+      </c>
+      <c r="M24" t="s">
+        <v>98</v>
+      </c>
+      <c r="N24" t="s">
+        <v>99</v>
+      </c>
+      <c r="O24" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B25" t="s">
+        <v>88</v>
+      </c>
+      <c r="C25" t="s">
+        <v>102</v>
+      </c>
+      <c r="D25" t="s">
         <v>103</v>
       </c>
-      <c r="I11" t="s">
+      <c r="E25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G25" t="s">
+        <v>88</v>
+      </c>
+      <c r="H25" t="s">
+        <v>102</v>
+      </c>
+      <c r="I25" t="s">
+        <v>103</v>
+      </c>
+      <c r="J25" t="s">
         <v>104</v>
       </c>
-      <c r="J11" t="s">
-        <v>111</v>
-      </c>
-      <c r="L11" t="s">
-        <v>87</v>
-      </c>
-      <c r="M11" t="s">
+      <c r="L25" t="s">
         <v>88</v>
       </c>
-      <c r="N11" t="s">
-        <v>89</v>
-      </c>
-      <c r="O11" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>87</v>
-      </c>
-      <c r="R11" t="s">
+      <c r="M25" t="s">
+        <v>100</v>
+      </c>
+      <c r="N25" t="s">
         <v>101</v>
       </c>
-      <c r="S11" t="s">
-        <v>102</v>
-      </c>
-      <c r="T11" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="B12" t="s">
-        <v>87</v>
-      </c>
-      <c r="C12" t="s">
-        <v>91</v>
-      </c>
-      <c r="D12" t="s">
-        <v>92</v>
-      </c>
-      <c r="E12" t="s">
-        <v>90</v>
-      </c>
-      <c r="G12" t="s">
-        <v>87</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="O25" t="s">
         <v>107</v>
       </c>
-      <c r="I12" t="s">
-        <v>108</v>
-      </c>
-      <c r="J12" t="s">
-        <v>111</v>
-      </c>
-      <c r="L12" t="s">
-        <v>87</v>
-      </c>
-      <c r="M12" t="s">
-        <v>91</v>
-      </c>
-      <c r="N12" t="s">
-        <v>92</v>
-      </c>
-      <c r="O12" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>87</v>
-      </c>
-      <c r="R12" t="s">
+    </row>
+    <row r="26" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="G26" t="s">
         <v>88</v>
       </c>
-      <c r="S12" t="s">
-        <v>89</v>
-      </c>
-      <c r="T12" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="B13" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" t="s">
-        <v>93</v>
-      </c>
-      <c r="D13" t="s">
-        <v>94</v>
-      </c>
-      <c r="E13" t="s">
-        <v>90</v>
-      </c>
-      <c r="G13" t="s">
-        <v>87</v>
-      </c>
-      <c r="H13" t="s">
-        <v>91</v>
-      </c>
-      <c r="I13" t="s">
-        <v>92</v>
-      </c>
-      <c r="J13" t="s">
-        <v>111</v>
-      </c>
-      <c r="L13" t="s">
-        <v>87</v>
-      </c>
-      <c r="M13" t="s">
-        <v>93</v>
-      </c>
-      <c r="N13" t="s">
-        <v>94</v>
-      </c>
-      <c r="O13" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>87</v>
-      </c>
-      <c r="R13" t="s">
-        <v>103</v>
-      </c>
-      <c r="S13" t="s">
+      <c r="H26" t="s">
+        <v>105</v>
+      </c>
+      <c r="I26" t="s">
+        <v>106</v>
+      </c>
+      <c r="J26" t="s">
         <v>104</v>
       </c>
-      <c r="T13" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="B14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C14" t="s">
-        <v>95</v>
-      </c>
-      <c r="D14" t="s">
-        <v>96</v>
-      </c>
-      <c r="E14" t="s">
-        <v>90</v>
-      </c>
-      <c r="G14" t="s">
-        <v>87</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="L26" t="s">
         <v>88</v>
       </c>
-      <c r="I14" t="s">
-        <v>89</v>
-      </c>
-      <c r="J14" t="s">
-        <v>111</v>
-      </c>
-      <c r="L14" t="s">
-        <v>87</v>
-      </c>
-      <c r="M14" t="s">
-        <v>95</v>
-      </c>
-      <c r="N14" t="s">
-        <v>96</v>
-      </c>
-      <c r="O14" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>87</v>
-      </c>
-      <c r="R14" t="s">
-        <v>97</v>
-      </c>
-      <c r="S14" t="s">
-        <v>98</v>
-      </c>
-      <c r="T14" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="B15" t="s">
-        <v>87</v>
-      </c>
-      <c r="C15" t="s">
-        <v>97</v>
-      </c>
-      <c r="D15" t="s">
-        <v>98</v>
-      </c>
-      <c r="E15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H15" t="s">
-        <v>97</v>
-      </c>
-      <c r="I15" t="s">
-        <v>98</v>
-      </c>
-      <c r="J15" t="s">
-        <v>111</v>
-      </c>
-      <c r="L15" t="s">
-        <v>87</v>
-      </c>
-      <c r="M15" t="s">
-        <v>97</v>
-      </c>
-      <c r="N15" t="s">
-        <v>98</v>
-      </c>
-      <c r="O15" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>87</v>
-      </c>
-      <c r="R15" t="s">
-        <v>91</v>
-      </c>
-      <c r="S15" t="s">
-        <v>92</v>
-      </c>
-      <c r="T15" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="B16" t="s">
-        <v>87</v>
-      </c>
-      <c r="C16" t="s">
-        <v>99</v>
-      </c>
-      <c r="D16" t="s">
-        <v>100</v>
-      </c>
-      <c r="E16" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" t="s">
-        <v>87</v>
-      </c>
-      <c r="H16" t="s">
-        <v>95</v>
-      </c>
-      <c r="I16" t="s">
-        <v>96</v>
-      </c>
-      <c r="J16" t="s">
-        <v>111</v>
-      </c>
-      <c r="L16" t="s">
-        <v>87</v>
-      </c>
-      <c r="M16" t="s">
-        <v>99</v>
-      </c>
-      <c r="N16" t="s">
-        <v>100</v>
-      </c>
-      <c r="O16" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>87</v>
-      </c>
-      <c r="R16" t="s">
-        <v>99</v>
-      </c>
-      <c r="S16" t="s">
-        <v>100</v>
-      </c>
-      <c r="T16" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="B17" t="s">
-        <v>87</v>
-      </c>
-      <c r="C17" t="s">
-        <v>101</v>
-      </c>
-      <c r="D17" t="s">
-        <v>102</v>
-      </c>
-      <c r="E17" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" t="s">
-        <v>87</v>
-      </c>
-      <c r="H17" t="s">
-        <v>99</v>
-      </c>
-      <c r="I17" t="s">
-        <v>100</v>
-      </c>
-      <c r="J17" t="s">
-        <v>111</v>
-      </c>
-      <c r="L17" t="s">
-        <v>87</v>
-      </c>
-      <c r="M17" t="s">
+      <c r="M26" t="s">
+        <v>105</v>
+      </c>
+      <c r="N26" t="s">
+        <v>106</v>
+      </c>
+      <c r="O26" t="s">
         <v>107</v>
-      </c>
-      <c r="N17" t="s">
-        <v>108</v>
-      </c>
-      <c r="O17" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>87</v>
-      </c>
-      <c r="R17" t="s">
-        <v>105</v>
-      </c>
-      <c r="S17" t="s">
-        <v>106</v>
-      </c>
-      <c r="T17" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="B18" t="s">
-        <v>87</v>
-      </c>
-      <c r="C18" t="s">
-        <v>103</v>
-      </c>
-      <c r="D18" t="s">
-        <v>104</v>
-      </c>
-      <c r="E18" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" t="s">
-        <v>87</v>
-      </c>
-      <c r="H18" t="s">
-        <v>109</v>
-      </c>
-      <c r="I18" t="s">
-        <v>110</v>
-      </c>
-      <c r="J18" t="s">
-        <v>111</v>
-      </c>
-      <c r="L18" t="s">
-        <v>87</v>
-      </c>
-      <c r="M18" t="s">
-        <v>103</v>
-      </c>
-      <c r="N18" t="s">
-        <v>104</v>
-      </c>
-      <c r="O18" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>87</v>
-      </c>
-      <c r="R18" t="s">
-        <v>95</v>
-      </c>
-      <c r="S18" t="s">
-        <v>96</v>
-      </c>
-      <c r="T18" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="19" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="B19" t="s">
-        <v>87</v>
-      </c>
-      <c r="C19" t="s">
-        <v>105</v>
-      </c>
-      <c r="D19" t="s">
-        <v>106</v>
-      </c>
-      <c r="E19" t="s">
-        <v>90</v>
-      </c>
-      <c r="G19" t="s">
-        <v>87</v>
-      </c>
-      <c r="H19" t="s">
-        <v>93</v>
-      </c>
-      <c r="I19" t="s">
-        <v>94</v>
-      </c>
-      <c r="J19" t="s">
-        <v>111</v>
-      </c>
-      <c r="L19" t="s">
-        <v>87</v>
-      </c>
-      <c r="M19" t="s">
-        <v>101</v>
-      </c>
-      <c r="N19" t="s">
-        <v>102</v>
-      </c>
-      <c r="O19" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q19" t="s">
-        <v>87</v>
-      </c>
-      <c r="R19" t="s">
-        <v>93</v>
-      </c>
-      <c r="S19" t="s">
-        <v>94</v>
-      </c>
-      <c r="T19" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="B20" t="s">
-        <v>87</v>
-      </c>
-      <c r="C20" t="s">
-        <v>107</v>
-      </c>
-      <c r="D20" t="s">
-        <v>108</v>
-      </c>
-      <c r="E20" t="s">
-        <v>90</v>
-      </c>
-      <c r="G20" t="s">
-        <v>87</v>
-      </c>
-      <c r="H20" t="s">
-        <v>105</v>
-      </c>
-      <c r="I20" t="s">
-        <v>106</v>
-      </c>
-      <c r="J20" t="s">
-        <v>111</v>
-      </c>
-      <c r="L20" t="s">
-        <v>87</v>
-      </c>
-      <c r="M20" t="s">
-        <v>105</v>
-      </c>
-      <c r="N20" t="s">
-        <v>106</v>
-      </c>
-      <c r="O20" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>87</v>
-      </c>
-      <c r="R20" t="s">
-        <v>107</v>
-      </c>
-      <c r="S20" t="s">
-        <v>108</v>
-      </c>
-      <c r="T20" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="B21" t="s">
-        <v>87</v>
-      </c>
-      <c r="C21" t="s">
-        <v>109</v>
-      </c>
-      <c r="D21" t="s">
-        <v>110</v>
-      </c>
-      <c r="E21" t="s">
-        <v>90</v>
-      </c>
-      <c r="G21" t="s">
-        <v>87</v>
-      </c>
-      <c r="H21" t="s">
-        <v>101</v>
-      </c>
-      <c r="I21" t="s">
-        <v>102</v>
-      </c>
-      <c r="J21" t="s">
-        <v>111</v>
-      </c>
-      <c r="L21" t="s">
-        <v>87</v>
-      </c>
-      <c r="M21" t="s">
-        <v>109</v>
-      </c>
-      <c r="N21" t="s">
-        <v>110</v>
-      </c>
-      <c r="O21" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -1976,7 +2082,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="C4:X57"/>
+  <dimension ref="C4:X58"/>
   <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="13.3984375" bestFit="1" customWidth="1"/>
@@ -2556,6 +2662,9 @@
       <c r="G28" t="s">
         <v>5</v>
       </c>
+      <c r="H28" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="29" spans="3:24" x14ac:dyDescent="0.45">
       <c r="C29" t="s">
@@ -2578,6 +2687,9 @@
       <c r="G30" s="1">
         <v>1</v>
       </c>
+      <c r="H30" s="3" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="31" spans="3:24" x14ac:dyDescent="0.45">
       <c r="C31" t="s">
@@ -2637,39 +2749,39 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.45">
-      <c r="C38" t="s">
-        <v>20</v>
+    <row r="36" spans="3:7" x14ac:dyDescent="0.45">
+      <c r="C36" t="s">
+        <v>53</v>
+      </c>
+      <c r="D36" t="s">
+        <v>84</v>
+      </c>
+      <c r="G36" s="1">
+        <v>0.9</v>
       </c>
     </row>
     <row r="39" spans="3:7" x14ac:dyDescent="0.45">
       <c r="C39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D39" t="s">
-        <v>22</v>
-      </c>
-      <c r="E39" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="3:7" x14ac:dyDescent="0.45">
       <c r="C40" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D40" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="E40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="41" spans="3:7" x14ac:dyDescent="0.45">
       <c r="C41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D41" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="E41" t="s">
         <v>24</v>
@@ -2677,10 +2789,10 @@
     </row>
     <row r="42" spans="3:7" x14ac:dyDescent="0.45">
       <c r="C42" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="D42" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="E42" t="s">
         <v>24</v>
@@ -2688,10 +2800,10 @@
     </row>
     <row r="43" spans="3:7" x14ac:dyDescent="0.45">
       <c r="C43" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D43" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="E43" t="s">
         <v>24</v>
@@ -2699,120 +2811,128 @@
     </row>
     <row r="44" spans="3:7" x14ac:dyDescent="0.45">
       <c r="C44" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D44" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E44" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="47" spans="3:7" x14ac:dyDescent="0.45">
-      <c r="C47" t="s">
-        <v>4</v>
+    <row r="45" spans="3:7" x14ac:dyDescent="0.45">
+      <c r="C45" t="s">
+        <v>56</v>
+      </c>
+      <c r="D45" t="s">
+        <v>73</v>
+      </c>
+      <c r="E45" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="48" spans="3:7" x14ac:dyDescent="0.45">
       <c r="C48" t="s">
-        <v>1</v>
-      </c>
-      <c r="D48" t="s">
-        <v>26</v>
-      </c>
-      <c r="E48" t="s">
-        <v>66</v>
-      </c>
-      <c r="F48" t="s">
-        <v>65</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="3:13" x14ac:dyDescent="0.45">
       <c r="C49" t="s">
-        <v>64</v>
-      </c>
-      <c r="D49">
-        <v>2025</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>67</v>
+        <v>1</v>
+      </c>
+      <c r="D49" t="s">
+        <v>26</v>
+      </c>
+      <c r="E49" t="s">
+        <v>66</v>
       </c>
       <c r="F49" t="s">
-        <v>68</v>
+        <v>108</v>
+      </c>
+      <c r="G49" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="50" spans="3:13" x14ac:dyDescent="0.45">
       <c r="C50" t="s">
+        <v>64</v>
+      </c>
+      <c r="D50">
+        <v>2025</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G50" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="51" spans="3:13" x14ac:dyDescent="0.45">
+      <c r="C51" t="s">
         <v>69</v>
       </c>
-      <c r="D50">
+      <c r="D51">
         <v>40</v>
       </c>
-      <c r="E50" s="3" t="s">
+      <c r="E51" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="F50" t="s">
+      <c r="G51" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="54" spans="3:13" x14ac:dyDescent="0.45">
-      <c r="C54" t="s">
-        <v>52</v>
+    <row r="52" spans="3:13" x14ac:dyDescent="0.45">
+      <c r="C52" t="s">
+        <v>64</v>
+      </c>
+      <c r="D52">
+        <v>2100</v>
+      </c>
+      <c r="F52" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="55" spans="3:13" x14ac:dyDescent="0.45">
       <c r="C55" t="s">
-        <v>25</v>
-      </c>
-      <c r="D55" t="s">
-        <v>75</v>
-      </c>
-      <c r="E55" t="s">
-        <v>65</v>
-      </c>
-      <c r="F55" t="s">
-        <v>21</v>
-      </c>
-      <c r="G55" t="s">
-        <v>66</v>
-      </c>
-      <c r="H55">
-        <v>0</v>
-      </c>
-      <c r="I55">
-        <v>2022</v>
-      </c>
-      <c r="J55">
-        <v>2030</v>
-      </c>
-      <c r="K55" t="s">
-        <v>76</v>
-      </c>
-      <c r="L55" t="s">
-        <v>77</v>
-      </c>
-      <c r="M55" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
     </row>
     <row r="56" spans="3:13" x14ac:dyDescent="0.45">
       <c r="C56" t="s">
-        <v>78</v>
+        <v>25</v>
+      </c>
+      <c r="D56" t="s">
+        <v>75</v>
       </c>
       <c r="E56" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="F56" t="s">
-        <v>82</v>
+        <v>21</v>
+      </c>
+      <c r="G56" t="s">
+        <v>66</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
       </c>
       <c r="I56">
-        <v>0.95</v>
+        <v>2022</v>
+      </c>
+      <c r="J56">
+        <v>2030</v>
+      </c>
+      <c r="K56" t="s">
+        <v>76</v>
       </c>
       <c r="L56" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="M56" t="s">
-        <v>81</v>
+        <v>22</v>
       </c>
     </row>
     <row r="57" spans="3:13" x14ac:dyDescent="0.45">
@@ -2820,18 +2940,38 @@
         <v>78</v>
       </c>
       <c r="E57" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F57" t="s">
         <v>82</v>
       </c>
       <c r="I57">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="L57" t="s">
         <v>80</v>
       </c>
       <c r="M57" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="58" spans="3:13" x14ac:dyDescent="0.45">
+      <c r="C58" t="s">
+        <v>78</v>
+      </c>
+      <c r="E58" t="s">
+        <v>83</v>
+      </c>
+      <c r="F58" t="s">
+        <v>82</v>
+      </c>
+      <c r="I58">
+        <v>0.85</v>
+      </c>
+      <c r="L58" t="s">
+        <v>80</v>
+      </c>
+      <c r="M58" t="s">
         <v>81</v>
       </c>
     </row>

</xml_diff>